<commit_message>
weight average destination grades by incoming payloads while updating its balance
</commit_message>
<xml_diff>
--- a/blendmaster_backend_OOP/output/report_data_2024-11-28_06-00.xlsx
+++ b/blendmaster_backend_OOP/output/report_data_2024-11-28_06-00.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster_backend_OOP\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26AC29C3-91DC-4186-92EF-87879C2BA471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C6BFD48-F43F-4554-9AC3-A64B6266A1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11430" yWindow="-21720" windowWidth="51840" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="47">
   <si>
     <t>start_datetime</t>
   </si>
@@ -139,25 +139,25 @@
     <t>preplan</t>
   </si>
   <si>
+    <t>CEN01_LT01_2002</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
     <t>CEN01_RP01_0104</t>
   </si>
   <si>
-    <t>RC</t>
-  </si>
-  <si>
-    <t>CEN01_RP01_0105</t>
-  </si>
-  <si>
     <t>CEN01_RP01_0106</t>
   </si>
   <si>
-    <t>ELW01_RP01_0222</t>
+    <t>CEN01_RP01_0109</t>
+  </si>
+  <si>
+    <t>ELW01_RP01_0807</t>
   </si>
   <si>
     <t>period_1</t>
-  </si>
-  <si>
-    <t>ELW01_RP01_0211</t>
   </si>
   <si>
     <t>period_2</t>
@@ -182,7 +182,6 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -528,7 +527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AL13"/>
+  <dimension ref="A1:AL16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="18.109375" bestFit="1" customWidth="1"/>
@@ -700,7 +699,7 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
         <v>12</v>
@@ -712,31 +711,31 @@
         <v>39</v>
       </c>
       <c r="I2">
-        <v>0.28999999999999998</v>
+        <v>0.25</v>
       </c>
       <c r="J2">
-        <v>366621.88949999999</v>
+        <v>190815.59999999989</v>
       </c>
       <c r="K2">
-        <v>12000</v>
+        <v>10440.30427210718</v>
       </c>
       <c r="L2">
-        <v>354621.88949999999</v>
+        <v>180375.29572789281</v>
       </c>
       <c r="M2">
-        <v>61.477307236232249</v>
+        <v>55.356930728690656</v>
       </c>
       <c r="N2">
-        <v>3.8636422713947809</v>
+        <v>7.9115042557894366</v>
       </c>
       <c r="O2">
-        <v>2.516706629273084</v>
+        <v>4.8007215415563369</v>
       </c>
       <c r="P2">
-        <v>0.1207421305527467</v>
+        <v>0.1323212982382439</v>
       </c>
       <c r="Q2">
-        <v>4.1509304680857478E-2</v>
+        <v>5.6638072117720852E-2</v>
       </c>
       <c r="R2" t="s">
         <v>40</v>
@@ -745,7 +744,7 @@
         <v>1000</v>
       </c>
       <c r="T2">
-        <v>1000</v>
+        <v>870.02535600893191</v>
       </c>
       <c r="U2">
         <v>42000</v>
@@ -757,19 +756,19 @@
         <v>3500</v>
       </c>
       <c r="X2">
-        <v>59.694009014360638</v>
+        <v>59.652466165742908</v>
       </c>
       <c r="Y2">
-        <v>4.9441981462439033</v>
+        <v>5</v>
       </c>
       <c r="Z2">
-        <v>2.7250288330696391</v>
+        <v>3</v>
       </c>
       <c r="AA2">
-        <v>0.1050708858159393</v>
+        <v>0.11949790430874049</v>
       </c>
       <c r="AB2">
-        <v>3.9822850093257131E-2</v>
+        <v>4.2313475389365029E-2</v>
       </c>
       <c r="AC2">
         <v>58.5</v>
@@ -816,7 +815,7 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3">
         <v>12</v>
@@ -828,31 +827,31 @@
         <v>41</v>
       </c>
       <c r="I3">
-        <v>0.28999999999999998</v>
+        <v>0.06</v>
       </c>
       <c r="J3">
-        <v>369144.38900000002</v>
+        <v>414990.772</v>
       </c>
       <c r="K3">
-        <v>12000</v>
+        <v>2525.0778580603628</v>
       </c>
       <c r="L3">
-        <v>357144.38900000002</v>
+        <v>412465.69414193957</v>
       </c>
       <c r="M3">
-        <v>59.580084798070871</v>
+        <v>61.308271104869071</v>
       </c>
       <c r="N3">
-        <v>5.2538880405507014</v>
+        <v>3.8377867085694479</v>
       </c>
       <c r="O3">
-        <v>2.368739705797716</v>
+        <v>2.585931121324168</v>
       </c>
       <c r="P3">
-        <v>0.11247771246205281</v>
+        <v>0.12271527936229989</v>
       </c>
       <c r="Q3">
-        <v>3.1749504113244877E-2</v>
+        <v>4.3146185628212E-2</v>
       </c>
       <c r="R3" t="s">
         <v>40</v>
@@ -861,7 +860,7 @@
         <v>1000</v>
       </c>
       <c r="T3">
-        <v>1000</v>
+        <v>210.42315483836359</v>
       </c>
       <c r="U3">
         <v>42000</v>
@@ -873,19 +872,19 @@
         <v>3500</v>
       </c>
       <c r="X3">
-        <v>59.694009014360638</v>
+        <v>59.652466165742908</v>
       </c>
       <c r="Y3">
-        <v>4.9441981462439033</v>
+        <v>5</v>
       </c>
       <c r="Z3">
-        <v>2.7250288330696391</v>
+        <v>3</v>
       </c>
       <c r="AA3">
-        <v>0.1050708858159393</v>
+        <v>0.11949790430874049</v>
       </c>
       <c r="AB3">
-        <v>3.9822850093257131E-2</v>
+        <v>4.2313475389365029E-2</v>
       </c>
       <c r="AC3">
         <v>58.5</v>
@@ -932,7 +931,7 @@
         <v>1</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4">
         <v>12</v>
@@ -947,28 +946,28 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="J4">
-        <v>89345</v>
+        <v>384942.95750000002</v>
       </c>
       <c r="K4">
         <v>12000</v>
       </c>
       <c r="L4">
-        <v>77345</v>
+        <v>372942.95750000002</v>
       </c>
       <c r="M4">
-        <v>59.883468563944113</v>
+        <v>60.778193732817833</v>
       </c>
       <c r="N4">
-        <v>4.1996001955675712</v>
+        <v>3.9124719303088331</v>
       </c>
       <c r="O4">
-        <v>2.8116592318517029</v>
+        <v>2.5433690830931228</v>
       </c>
       <c r="P4">
-        <v>0.10735070156647319</v>
+        <v>0.1143836194853638</v>
       </c>
       <c r="Q4">
-        <v>4.7718262790655337E-2</v>
+        <v>3.9630920120378013E-2</v>
       </c>
       <c r="R4" t="s">
         <v>40</v>
@@ -989,19 +988,19 @@
         <v>3500</v>
       </c>
       <c r="X4">
-        <v>59.694009014360638</v>
+        <v>59.652466165742908</v>
       </c>
       <c r="Y4">
-        <v>4.9441981462439033</v>
+        <v>5</v>
       </c>
       <c r="Z4">
-        <v>2.7250288330696391</v>
+        <v>3</v>
       </c>
       <c r="AA4">
-        <v>0.1050708858159393</v>
+        <v>0.11949790430874049</v>
       </c>
       <c r="AB4">
-        <v>3.9822850093257131E-2</v>
+        <v>4.2313475389365029E-2</v>
       </c>
       <c r="AC4">
         <v>58.5</v>
@@ -1048,7 +1047,7 @@
         <v>1</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5">
         <v>12</v>
@@ -1060,31 +1059,31 @@
         <v>43</v>
       </c>
       <c r="I5">
-        <v>0.14000000000000001</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="J5">
-        <v>21913.954719999991</v>
+        <v>313043.59875</v>
       </c>
       <c r="K5">
-        <v>6000</v>
+        <v>12000</v>
       </c>
       <c r="L5">
-        <v>15913.954719999991</v>
+        <v>301043.59875</v>
       </c>
       <c r="M5">
-        <v>55.976341904030001</v>
+        <v>61.795492014279141</v>
       </c>
       <c r="N5">
-        <v>7.9751260086812197</v>
+        <v>3.9093537543977188</v>
       </c>
       <c r="O5">
-        <v>3.680990697642466</v>
+        <v>2.3062204770750121</v>
       </c>
       <c r="P5">
-        <v>5.4355111549029819E-2</v>
+        <v>0.1221413849964776</v>
       </c>
       <c r="Q5">
-        <v>3.6805807483284471E-2</v>
+        <v>3.6055612168878759E-2</v>
       </c>
       <c r="R5" t="s">
         <v>40</v>
@@ -1093,7 +1092,7 @@
         <v>1000</v>
       </c>
       <c r="T5">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="U5">
         <v>42000</v>
@@ -1105,19 +1104,19 @@
         <v>3500</v>
       </c>
       <c r="X5">
-        <v>59.694009014360638</v>
+        <v>59.652466165742908</v>
       </c>
       <c r="Y5">
-        <v>4.9441981462439033</v>
+        <v>5</v>
       </c>
       <c r="Z5">
-        <v>2.7250288330696391</v>
+        <v>3</v>
       </c>
       <c r="AA5">
-        <v>0.1050708858159393</v>
+        <v>0.11949790430874049</v>
       </c>
       <c r="AB5">
-        <v>3.9822850093257131E-2</v>
+        <v>4.2313475389365029E-2</v>
       </c>
       <c r="AC5">
         <v>58.5</v>
@@ -1152,13 +1151,13 @@
     </row>
     <row r="6" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
+        <v>45624.25</v>
+      </c>
+      <c r="B6" s="2">
         <v>45624.75</v>
       </c>
-      <c r="B6" s="2">
-        <v>45625.25</v>
-      </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1170,37 +1169,37 @@
         <v>12</v>
       </c>
       <c r="G6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" t="s">
         <v>44</v>
       </c>
-      <c r="H6" t="s">
-        <v>39</v>
-      </c>
       <c r="I6">
-        <v>0.28999999999999998</v>
+        <v>0.12</v>
       </c>
       <c r="J6">
-        <v>354621.88949999999</v>
+        <v>26544.616000000002</v>
       </c>
       <c r="K6">
-        <v>12000</v>
+        <v>5034.6178698324529</v>
       </c>
       <c r="L6">
-        <v>342621.88949999999</v>
+        <v>21509.998130167551</v>
       </c>
       <c r="M6">
-        <v>61.477307236232249</v>
+        <v>59.938608954590642</v>
       </c>
       <c r="N6">
-        <v>3.8636422713947809</v>
+        <v>4.7369771605000368</v>
       </c>
       <c r="O6">
-        <v>2.516706629273084</v>
+        <v>2.2155115899433908</v>
       </c>
       <c r="P6">
-        <v>0.1207421305527467</v>
+        <v>9.718149217754718E-2</v>
       </c>
       <c r="Q6">
-        <v>4.1509304680857478E-2</v>
+        <v>3.35003368594778E-2</v>
       </c>
       <c r="R6" t="s">
         <v>40</v>
@@ -1209,7 +1208,7 @@
         <v>1000</v>
       </c>
       <c r="T6">
-        <v>1000</v>
+        <v>419.55148915270439</v>
       </c>
       <c r="U6">
         <v>42000</v>
@@ -1221,19 +1220,19 @@
         <v>3500</v>
       </c>
       <c r="X6">
-        <v>60.254651240041582</v>
+        <v>59.652466165742908</v>
       </c>
       <c r="Y6">
-        <v>4.4868413517184127</v>
+        <v>5</v>
       </c>
       <c r="Z6">
-        <v>2.600739698784337</v>
+        <v>3</v>
       </c>
       <c r="AA6">
-        <v>0.11590017345970589</v>
+        <v>0.11949790430874049</v>
       </c>
       <c r="AB6">
-        <v>4.960808311595772E-2</v>
+        <v>4.2313475389365029E-2</v>
       </c>
       <c r="AC6">
         <v>58.5</v>
@@ -1286,37 +1285,37 @@
         <v>12</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I7">
-        <v>0.28999999999999998</v>
+        <v>0.25</v>
       </c>
       <c r="J7">
-        <v>357144.38900000002</v>
+        <v>180375.29572789281</v>
       </c>
       <c r="K7">
-        <v>12000</v>
+        <v>10440.30427210718</v>
       </c>
       <c r="L7">
-        <v>345144.38900000002</v>
+        <v>169934.99145578561</v>
       </c>
       <c r="M7">
-        <v>59.580084798070871</v>
+        <v>55.356930728690656</v>
       </c>
       <c r="N7">
-        <v>5.2538880405507014</v>
+        <v>7.9115042557894366</v>
       </c>
       <c r="O7">
-        <v>2.368739705797716</v>
+        <v>4.8007215415563369</v>
       </c>
       <c r="P7">
-        <v>0.11247771246205281</v>
+        <v>0.1323212982382439</v>
       </c>
       <c r="Q7">
-        <v>3.1749504113244877E-2</v>
+        <v>5.6638072117720852E-2</v>
       </c>
       <c r="R7" t="s">
         <v>40</v>
@@ -1325,7 +1324,7 @@
         <v>1000</v>
       </c>
       <c r="T7">
-        <v>1000</v>
+        <v>870.02535600893191</v>
       </c>
       <c r="U7">
         <v>42000</v>
@@ -1337,19 +1336,19 @@
         <v>3500</v>
       </c>
       <c r="X7">
-        <v>60.254651240041582</v>
+        <v>59.652466165742908</v>
       </c>
       <c r="Y7">
-        <v>4.4868413517184127</v>
+        <v>5</v>
       </c>
       <c r="Z7">
-        <v>2.600739698784337</v>
+        <v>3</v>
       </c>
       <c r="AA7">
-        <v>0.11590017345970589</v>
+        <v>0.11949790430874049</v>
       </c>
       <c r="AB7">
-        <v>4.960808311595772E-2</v>
+        <v>4.2313475389365029E-2</v>
       </c>
       <c r="AC7">
         <v>58.5</v>
@@ -1402,37 +1401,37 @@
         <v>12</v>
       </c>
       <c r="G8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I8">
-        <v>0.28999999999999998</v>
+        <v>0.06</v>
       </c>
       <c r="J8">
-        <v>85382.379534623557</v>
+        <v>412465.69414193957</v>
       </c>
       <c r="K8">
-        <v>12000</v>
+        <v>2525.0778580603628</v>
       </c>
       <c r="L8">
-        <v>73382.379534623557</v>
+        <v>409940.61628387932</v>
       </c>
       <c r="M8">
-        <v>59.883468563944113</v>
+        <v>61.308271104869071</v>
       </c>
       <c r="N8">
-        <v>4.1996001955675712</v>
+        <v>3.8377867085694479</v>
       </c>
       <c r="O8">
-        <v>2.8116592318517029</v>
+        <v>2.585931121324168</v>
       </c>
       <c r="P8">
-        <v>0.10735070156647319</v>
+        <v>0.12271527936229989</v>
       </c>
       <c r="Q8">
-        <v>4.7718262790655337E-2</v>
+        <v>4.3146185628212E-2</v>
       </c>
       <c r="R8" t="s">
         <v>40</v>
@@ -1441,7 +1440,7 @@
         <v>1000</v>
       </c>
       <c r="T8">
-        <v>1000</v>
+        <v>210.42315483836359</v>
       </c>
       <c r="U8">
         <v>42000</v>
@@ -1453,19 +1452,19 @@
         <v>3500</v>
       </c>
       <c r="X8">
-        <v>60.254651240041582</v>
+        <v>59.652466165742908</v>
       </c>
       <c r="Y8">
-        <v>4.4868413517184127</v>
+        <v>5</v>
       </c>
       <c r="Z8">
-        <v>2.600739698784337</v>
+        <v>3</v>
       </c>
       <c r="AA8">
-        <v>0.11590017345970589</v>
+        <v>0.11949790430874049</v>
       </c>
       <c r="AB8">
-        <v>4.960808311595772E-2</v>
+        <v>4.2313475389365029E-2</v>
       </c>
       <c r="AC8">
         <v>58.5</v>
@@ -1518,37 +1517,37 @@
         <v>12</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I9">
-        <v>0.14000000000000001</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="J9">
-        <v>69487.741750000001</v>
+        <v>380980.33703462349</v>
       </c>
       <c r="K9">
-        <v>6000</v>
+        <v>12000</v>
       </c>
       <c r="L9">
-        <v>63487.741750000001</v>
+        <v>368980.33703462349</v>
       </c>
       <c r="M9">
-        <v>59.900837483796622</v>
+        <v>60.778193732817833</v>
       </c>
       <c r="N9">
-        <v>4.7736284470027837</v>
+        <v>3.9124719303088331</v>
       </c>
       <c r="O9">
-        <v>2.810966757645355</v>
+        <v>2.5433690830931228</v>
       </c>
       <c r="P9">
-        <v>0.1301601250553964</v>
+        <v>0.1143836194853638</v>
       </c>
       <c r="Q9">
-        <v>0.10530243864218861</v>
+        <v>3.9630920120378013E-2</v>
       </c>
       <c r="R9" t="s">
         <v>40</v>
@@ -1557,7 +1556,7 @@
         <v>1000</v>
       </c>
       <c r="T9">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="U9">
         <v>42000</v>
@@ -1569,19 +1568,19 @@
         <v>3500</v>
       </c>
       <c r="X9">
-        <v>60.254651240041582</v>
+        <v>59.652466165742908</v>
       </c>
       <c r="Y9">
-        <v>4.4868413517184127</v>
+        <v>5</v>
       </c>
       <c r="Z9">
-        <v>2.600739698784337</v>
+        <v>3</v>
       </c>
       <c r="AA9">
-        <v>0.11590017345970589</v>
+        <v>0.11949790430874049</v>
       </c>
       <c r="AB9">
-        <v>4.960808311595772E-2</v>
+        <v>4.2313475389365029E-2</v>
       </c>
       <c r="AC9">
         <v>58.5</v>
@@ -1616,55 +1615,55 @@
     </row>
     <row r="10" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
+        <v>45624.75</v>
+      </c>
+      <c r="B10" s="2">
         <v>45625.25</v>
       </c>
-      <c r="B10" s="2">
-        <v>45625.75</v>
-      </c>
       <c r="C10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10">
         <v>12</v>
       </c>
       <c r="G10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H10" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I10">
         <v>0.28999999999999998</v>
       </c>
       <c r="J10">
-        <v>342621.88949999999</v>
+        <v>301043.59875</v>
       </c>
       <c r="K10">
         <v>12000</v>
       </c>
       <c r="L10">
-        <v>330621.88949999999</v>
+        <v>289043.59875</v>
       </c>
       <c r="M10">
-        <v>61.477307236232249</v>
+        <v>61.795492014279141</v>
       </c>
       <c r="N10">
-        <v>3.8636422713947809</v>
+        <v>3.9093537543977188</v>
       </c>
       <c r="O10">
-        <v>2.516706629273084</v>
+        <v>2.3062204770750121</v>
       </c>
       <c r="P10">
-        <v>0.1207421305527467</v>
+        <v>0.1221413849964776</v>
       </c>
       <c r="Q10">
-        <v>4.1509304680857478E-2</v>
+        <v>3.6055612168878759E-2</v>
       </c>
       <c r="R10" t="s">
         <v>40</v>
@@ -1685,19 +1684,19 @@
         <v>3500</v>
       </c>
       <c r="X10">
-        <v>59.694009014360638</v>
+        <v>59.652466165742908</v>
       </c>
       <c r="Y10">
-        <v>4.9441981462439033</v>
+        <v>5</v>
       </c>
       <c r="Z10">
-        <v>2.7250288330696391</v>
+        <v>3</v>
       </c>
       <c r="AA10">
-        <v>0.1050708858159393</v>
+        <v>0.11949790430874049</v>
       </c>
       <c r="AB10">
-        <v>3.9822850093257131E-2</v>
+        <v>4.2313475389365029E-2</v>
       </c>
       <c r="AC10">
         <v>58.5</v>
@@ -1732,55 +1731,55 @@
     </row>
     <row r="11" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
+        <v>45624.75</v>
+      </c>
+      <c r="B11" s="2">
         <v>45625.25</v>
       </c>
-      <c r="B11" s="2">
-        <v>45625.75</v>
-      </c>
       <c r="C11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11">
         <v>1</v>
       </c>
       <c r="E11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11">
         <v>12</v>
       </c>
       <c r="G11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H11" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="I11">
-        <v>0.28999999999999998</v>
+        <v>0.12</v>
       </c>
       <c r="J11">
-        <v>345144.38900000002</v>
+        <v>21509.998130167551</v>
       </c>
       <c r="K11">
-        <v>12000</v>
+        <v>5034.6178698324529</v>
       </c>
       <c r="L11">
-        <v>333144.38900000002</v>
+        <v>16475.3802603351</v>
       </c>
       <c r="M11">
-        <v>59.580084798070871</v>
+        <v>59.938608954590642</v>
       </c>
       <c r="N11">
-        <v>5.2538880405507014</v>
+        <v>4.7369771605000368</v>
       </c>
       <c r="O11">
-        <v>2.368739705797716</v>
+        <v>2.2155115899433908</v>
       </c>
       <c r="P11">
-        <v>0.11247771246205281</v>
+        <v>9.718149217754718E-2</v>
       </c>
       <c r="Q11">
-        <v>3.1749504113244877E-2</v>
+        <v>3.35003368594778E-2</v>
       </c>
       <c r="R11" t="s">
         <v>40</v>
@@ -1789,7 +1788,7 @@
         <v>1000</v>
       </c>
       <c r="T11">
-        <v>1000</v>
+        <v>419.55148915270439</v>
       </c>
       <c r="U11">
         <v>42000</v>
@@ -1801,19 +1800,19 @@
         <v>3500</v>
       </c>
       <c r="X11">
-        <v>59.694009014360638</v>
+        <v>59.652466165742908</v>
       </c>
       <c r="Y11">
-        <v>4.9441981462439033</v>
+        <v>5</v>
       </c>
       <c r="Z11">
-        <v>2.7250288330696391</v>
+        <v>3</v>
       </c>
       <c r="AA11">
-        <v>0.1050708858159393</v>
+        <v>0.11949790430874049</v>
       </c>
       <c r="AB11">
-        <v>3.9822850093257131E-2</v>
+        <v>4.2313475389365029E-2</v>
       </c>
       <c r="AC11">
         <v>58.5</v>
@@ -1860,7 +1859,7 @@
         <v>1</v>
       </c>
       <c r="E12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12">
         <v>12</v>
@@ -1869,34 +1868,34 @@
         <v>46</v>
       </c>
       <c r="H12" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="I12">
-        <v>0.28999999999999998</v>
+        <v>0.25</v>
       </c>
       <c r="J12">
-        <v>109175.23471760729</v>
+        <v>169934.99145578561</v>
       </c>
       <c r="K12">
-        <v>12000</v>
+        <v>10440.30427210718</v>
       </c>
       <c r="L12">
-        <v>97175.234717607324</v>
+        <v>159494.68718367841</v>
       </c>
       <c r="M12">
-        <v>59.883468563944113</v>
+        <v>55.356930728690656</v>
       </c>
       <c r="N12">
-        <v>4.1996001955675712</v>
+        <v>7.9115042557894366</v>
       </c>
       <c r="O12">
-        <v>2.8116592318517029</v>
+        <v>4.8007215415563369</v>
       </c>
       <c r="P12">
-        <v>0.10735070156647319</v>
+        <v>0.1323212982382439</v>
       </c>
       <c r="Q12">
-        <v>4.7718262790655337E-2</v>
+        <v>5.6638072117720852E-2</v>
       </c>
       <c r="R12" t="s">
         <v>40</v>
@@ -1905,7 +1904,7 @@
         <v>1000</v>
       </c>
       <c r="T12">
-        <v>1000</v>
+        <v>870.02535600893191</v>
       </c>
       <c r="U12">
         <v>42000</v>
@@ -1917,19 +1916,19 @@
         <v>3500</v>
       </c>
       <c r="X12">
-        <v>59.694009014360638</v>
+        <v>59.652466165742908</v>
       </c>
       <c r="Y12">
-        <v>4.9441981462439033</v>
+        <v>5</v>
       </c>
       <c r="Z12">
-        <v>2.7250288330696391</v>
+        <v>3</v>
       </c>
       <c r="AA12">
-        <v>0.1050708858159393</v>
+        <v>0.11949790430874049</v>
       </c>
       <c r="AB12">
-        <v>3.9822850093257131E-2</v>
+        <v>4.2313475389365029E-2</v>
       </c>
       <c r="AC12">
         <v>58.5</v>
@@ -1976,7 +1975,7 @@
         <v>1</v>
       </c>
       <c r="E13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13">
         <v>12</v>
@@ -1985,34 +1984,34 @@
         <v>46</v>
       </c>
       <c r="H13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I13">
-        <v>0.14000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="J13">
-        <v>15913.954719999991</v>
+        <v>409940.61628387932</v>
       </c>
       <c r="K13">
-        <v>6000</v>
+        <v>2525.0778580603628</v>
       </c>
       <c r="L13">
-        <v>9913.9547199999943</v>
+        <v>407415.5384258189</v>
       </c>
       <c r="M13">
-        <v>55.976341904030001</v>
+        <v>61.308271104869071</v>
       </c>
       <c r="N13">
-        <v>7.9751260086812197</v>
+        <v>3.8377867085694479</v>
       </c>
       <c r="O13">
-        <v>3.680990697642466</v>
+        <v>2.585931121324168</v>
       </c>
       <c r="P13">
-        <v>5.4355111549029819E-2</v>
+        <v>0.12271527936229989</v>
       </c>
       <c r="Q13">
-        <v>3.6805807483284471E-2</v>
+        <v>4.3146185628212E-2</v>
       </c>
       <c r="R13" t="s">
         <v>40</v>
@@ -2021,7 +2020,7 @@
         <v>1000</v>
       </c>
       <c r="T13">
-        <v>500</v>
+        <v>210.42315483836359</v>
       </c>
       <c r="U13">
         <v>42000</v>
@@ -2033,19 +2032,19 @@
         <v>3500</v>
       </c>
       <c r="X13">
-        <v>59.694009014360638</v>
+        <v>59.652466165742908</v>
       </c>
       <c r="Y13">
-        <v>4.9441981462439033</v>
+        <v>5</v>
       </c>
       <c r="Z13">
-        <v>2.7250288330696391</v>
+        <v>3</v>
       </c>
       <c r="AA13">
-        <v>0.1050708858159393</v>
+        <v>0.11949790430874049</v>
       </c>
       <c r="AB13">
-        <v>3.9822850093257131E-2</v>
+        <v>4.2313475389365029E-2</v>
       </c>
       <c r="AC13">
         <v>58.5</v>
@@ -2075,6 +2074,354 @@
         <v>0</v>
       </c>
       <c r="AL13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
+        <v>45625.25</v>
+      </c>
+      <c r="B14" s="2">
+        <v>45625.75</v>
+      </c>
+      <c r="C14">
+        <v>2</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>2</v>
+      </c>
+      <c r="F14">
+        <v>12</v>
+      </c>
+      <c r="G14" t="s">
+        <v>46</v>
+      </c>
+      <c r="H14" t="s">
+        <v>42</v>
+      </c>
+      <c r="I14">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="J14">
+        <v>404773.19221760728</v>
+      </c>
+      <c r="K14">
+        <v>12000</v>
+      </c>
+      <c r="L14">
+        <v>392773.19221760728</v>
+      </c>
+      <c r="M14">
+        <v>60.778193732817833</v>
+      </c>
+      <c r="N14">
+        <v>3.9124719303088331</v>
+      </c>
+      <c r="O14">
+        <v>2.5433690830931228</v>
+      </c>
+      <c r="P14">
+        <v>0.1143836194853638</v>
+      </c>
+      <c r="Q14">
+        <v>3.9630920120378013E-2</v>
+      </c>
+      <c r="R14" t="s">
+        <v>40</v>
+      </c>
+      <c r="S14">
+        <v>1000</v>
+      </c>
+      <c r="T14">
+        <v>1000</v>
+      </c>
+      <c r="U14">
+        <v>42000</v>
+      </c>
+      <c r="V14">
+        <v>3500</v>
+      </c>
+      <c r="W14">
+        <v>3500</v>
+      </c>
+      <c r="X14">
+        <v>59.652466165742908</v>
+      </c>
+      <c r="Y14">
+        <v>5</v>
+      </c>
+      <c r="Z14">
+        <v>3</v>
+      </c>
+      <c r="AA14">
+        <v>0.11949790430874049</v>
+      </c>
+      <c r="AB14">
+        <v>4.2313475389365029E-2</v>
+      </c>
+      <c r="AC14">
+        <v>58.5</v>
+      </c>
+      <c r="AD14">
+        <v>61</v>
+      </c>
+      <c r="AE14">
+        <v>0</v>
+      </c>
+      <c r="AF14">
+        <v>5</v>
+      </c>
+      <c r="AG14">
+        <v>0</v>
+      </c>
+      <c r="AH14">
+        <v>3</v>
+      </c>
+      <c r="AI14">
+        <v>0</v>
+      </c>
+      <c r="AJ14">
+        <v>2</v>
+      </c>
+      <c r="AK14">
+        <v>0</v>
+      </c>
+      <c r="AL14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
+        <v>45625.25</v>
+      </c>
+      <c r="B15" s="2">
+        <v>45625.75</v>
+      </c>
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>2</v>
+      </c>
+      <c r="F15">
+        <v>12</v>
+      </c>
+      <c r="G15" t="s">
+        <v>46</v>
+      </c>
+      <c r="H15" t="s">
+        <v>43</v>
+      </c>
+      <c r="I15">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="J15">
+        <v>289043.59875</v>
+      </c>
+      <c r="K15">
+        <v>12000</v>
+      </c>
+      <c r="L15">
+        <v>277043.59875</v>
+      </c>
+      <c r="M15">
+        <v>61.795492014279141</v>
+      </c>
+      <c r="N15">
+        <v>3.9093537543977188</v>
+      </c>
+      <c r="O15">
+        <v>2.3062204770750121</v>
+      </c>
+      <c r="P15">
+        <v>0.1221413849964776</v>
+      </c>
+      <c r="Q15">
+        <v>3.6055612168878759E-2</v>
+      </c>
+      <c r="R15" t="s">
+        <v>40</v>
+      </c>
+      <c r="S15">
+        <v>1000</v>
+      </c>
+      <c r="T15">
+        <v>1000</v>
+      </c>
+      <c r="U15">
+        <v>42000</v>
+      </c>
+      <c r="V15">
+        <v>3500</v>
+      </c>
+      <c r="W15">
+        <v>3500</v>
+      </c>
+      <c r="X15">
+        <v>59.652466165742908</v>
+      </c>
+      <c r="Y15">
+        <v>5</v>
+      </c>
+      <c r="Z15">
+        <v>3</v>
+      </c>
+      <c r="AA15">
+        <v>0.11949790430874049</v>
+      </c>
+      <c r="AB15">
+        <v>4.2313475389365029E-2</v>
+      </c>
+      <c r="AC15">
+        <v>58.5</v>
+      </c>
+      <c r="AD15">
+        <v>61</v>
+      </c>
+      <c r="AE15">
+        <v>0</v>
+      </c>
+      <c r="AF15">
+        <v>5</v>
+      </c>
+      <c r="AG15">
+        <v>0</v>
+      </c>
+      <c r="AH15">
+        <v>3</v>
+      </c>
+      <c r="AI15">
+        <v>0</v>
+      </c>
+      <c r="AJ15">
+        <v>2</v>
+      </c>
+      <c r="AK15">
+        <v>0</v>
+      </c>
+      <c r="AL15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A16" s="2">
+        <v>45625.25</v>
+      </c>
+      <c r="B16" s="2">
+        <v>45625.75</v>
+      </c>
+      <c r="C16">
+        <v>2</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>2</v>
+      </c>
+      <c r="F16">
+        <v>12</v>
+      </c>
+      <c r="G16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H16" t="s">
+        <v>44</v>
+      </c>
+      <c r="I16">
+        <v>0.12</v>
+      </c>
+      <c r="J16">
+        <v>16475.3802603351</v>
+      </c>
+      <c r="K16">
+        <v>5034.6178698324529</v>
+      </c>
+      <c r="L16">
+        <v>11440.76239050265</v>
+      </c>
+      <c r="M16">
+        <v>59.938608954590642</v>
+      </c>
+      <c r="N16">
+        <v>4.7369771605000368</v>
+      </c>
+      <c r="O16">
+        <v>2.2155115899433908</v>
+      </c>
+      <c r="P16">
+        <v>9.718149217754718E-2</v>
+      </c>
+      <c r="Q16">
+        <v>3.35003368594778E-2</v>
+      </c>
+      <c r="R16" t="s">
+        <v>40</v>
+      </c>
+      <c r="S16">
+        <v>1000</v>
+      </c>
+      <c r="T16">
+        <v>419.55148915270439</v>
+      </c>
+      <c r="U16">
+        <v>42000</v>
+      </c>
+      <c r="V16">
+        <v>3500</v>
+      </c>
+      <c r="W16">
+        <v>3500</v>
+      </c>
+      <c r="X16">
+        <v>59.652466165742908</v>
+      </c>
+      <c r="Y16">
+        <v>5</v>
+      </c>
+      <c r="Z16">
+        <v>3</v>
+      </c>
+      <c r="AA16">
+        <v>0.11949790430874049</v>
+      </c>
+      <c r="AB16">
+        <v>4.2313475389365029E-2</v>
+      </c>
+      <c r="AC16">
+        <v>58.5</v>
+      </c>
+      <c r="AD16">
+        <v>61</v>
+      </c>
+      <c r="AE16">
+        <v>0</v>
+      </c>
+      <c r="AF16">
+        <v>5</v>
+      </c>
+      <c r="AG16">
+        <v>0</v>
+      </c>
+      <c r="AH16">
+        <v>3</v>
+      </c>
+      <c r="AI16">
+        <v>0</v>
+      </c>
+      <c r="AJ16">
+        <v>2</v>
+      </c>
+      <c r="AK16">
+        <v>0</v>
+      </c>
+      <c r="AL16">
         <v>2</v>
       </c>
     </row>

</xml_diff>